<commit_message>
FP&A Pack V2: comparativo LY, puente PVM, drill-down clientes y SKUs
</commit_message>
<xml_diff>
--- a/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
+++ b/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
@@ -15,7 +15,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BRIDGE" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX_FORECAST" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DICC" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMP_LY" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUENTE_VENTAS" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRILL_CLIENTES" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRILL_SKUS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DICC" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -495,7 +499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -567,12 +571,40 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>FX_FORECAST: exposición USD, sensibilidad y forecast FY con plan de acción</t>
+          <t>COMP_LY: H1-2025 vs H1-2026 like-for-like + canales YoY</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>PUENTE_VENTAS: volumen, precio, mix y descuento (atribuye los -1.70M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>DRILL_CLIENTES: CxC institucional por cliente y aging, con DSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>DRILL_SKUS: inventarios Hogar por SKU, valorizado y cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>FX_FORECAST: exposición USD, sensibilidad y forecast FY con plan de acción</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>DICC: diccionario de campos y linaje</t>
         </is>
@@ -584,6 +616,992 @@
     <mergeCell ref="A1"/>
     <mergeCell ref="A4"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Paso</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Monto (S/)</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Acumulado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>Ventas ppto</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="n">
+        <v>30100000</v>
+      </c>
+      <c r="C2" s="12" t="n">
+        <v>30100000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Efecto volumen</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>-1100000</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>29000000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Efecto precio (+2% lista parcial)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>29250000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Efecto mix canal/linea</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>-450000</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>28800000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Descuento comercial defensivo</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>-400000</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>28400000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>Ventas real H1</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>28400000</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>28400000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Drill-down cobranza — CxC Institucional S/ 2.00M por cliente y aging (S/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Cliente</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Corriente</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>31-60</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>61-90</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>90+</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>DSO (d)</t>
+        </is>
+      </c>
+      <c r="H2" s="10" t="inlineStr">
+        <is>
+          <t>Mora 60+</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Municipalidad de San Juan</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>300000</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D3" s="9" t="n">
+        <v>70000</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="12">
+        <f>SUM(B3:E3)</f>
+        <v/>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="H3" s="9">
+        <f>D3+E3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Red Salud Norte</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>120000</v>
+      </c>
+      <c r="D4" s="9" t="n">
+        <v>60000</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F4" s="12">
+        <f>SUM(B4:E4)</f>
+        <v/>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H4" s="9">
+        <f>D4+E4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>EduCorp S.A.</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>80000</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="12">
+        <f>SUM(B5:E5)</f>
+        <v/>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="H5" s="9">
+        <f>D5+E5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Minera Cascajal</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>280000</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="12">
+        <f>SUM(B6:E6)</f>
+        <v/>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H6" s="9">
+        <f>D6+E6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Agroindustrial del Valle</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C7" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="12">
+        <f>SUM(B7:E7)</f>
+        <v/>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="H7" s="9">
+        <f>D7+E7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Constructora VialSur</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>40000</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F8" s="12">
+        <f>SUM(B8:E8)</f>
+        <v/>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H8" s="9">
+        <f>D8+E8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Gobierno Regional</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>40000</v>
+      </c>
+      <c r="F9" s="12">
+        <f>SUM(B9:E9)</f>
+        <v/>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="H9" s="9">
+        <f>D9+E9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Otros menores</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>30000</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>20000</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="12">
+        <f>SUM(B10:E10)</f>
+        <v/>
+      </c>
+      <c r="G10" s="15" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="H10" s="9">
+        <f>D10+E10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B11" s="12">
+        <f>SUM(B3:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="12">
+        <f>SUM(C3:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="12">
+        <f>SUM(D3:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="12">
+        <f>SUM(E3:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="12">
+        <f>SUM(F3:F10)</f>
+        <v/>
+      </c>
+      <c r="H11" s="12">
+        <f>SUM(H3:H10)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Drill-down inventarios — linea Hogar S/ 3.35M por SKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Descripcion</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Stock (u)</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Costo u</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Valorizado</t>
+        </is>
+      </c>
+      <c r="F2" s="10" t="inlineStr">
+        <is>
+          <t>Vta/mes (u)</t>
+        </is>
+      </c>
+      <c r="G2" s="10" t="inlineStr">
+        <is>
+          <t>Cobertura (m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>HOG-014</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Detergente industrial 20kg</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n">
+        <v>14000</v>
+      </c>
+      <c r="D3" s="6" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="E3" s="9" t="n">
+        <v>259000</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G3" s="15" t="n">
+        <v>4.4</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>HOG-022</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Jabon liquido 5L</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="n">
+        <v>22000</v>
+      </c>
+      <c r="D4" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="E4" s="9" t="n">
+        <v>281600</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>4800</v>
+      </c>
+      <c r="G4" s="15" t="n">
+        <v>4.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>HOG-031</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Papel toalla x12</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="E5" s="9" t="n">
+        <v>282000</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>7500</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>HOG-007</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Desinfectante 1L</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="E6" s="9" t="n">
+        <v>189000</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>12000</v>
+      </c>
+      <c r="G6" s="15" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>HOG-045</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Escobas premium</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>18000</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="E7" s="9" t="n">
+        <v>124200</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G7" s="15" t="n">
+        <v>8.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>HOG-046</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Trapeadores</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>25000</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="E8" s="9" t="n">
+        <v>140000</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G8" s="15" t="n">
+        <v>8.300000000000001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>HOG-052</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Bolsas basura 100L x50</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="E9" s="9" t="n">
+        <v>438000</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G9" s="15" t="n">
+        <v>6.7</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>HOG-RESTO</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Resto linea Hogar (agregado)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="12" t="n">
+        <v>1636200</v>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="15" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="E11" s="12">
+        <f>SUM(E3:E10)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Campo</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>Definición</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>Origen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="16" t="inlineStr">
+        <is>
+          <t>Ventas netas</t>
+        </is>
+      </c>
+      <c r="B2" s="16" t="inlineStr">
+        <is>
+          <t>Ventas brutas menos devoluciones y descuentos</t>
+        </is>
+      </c>
+      <c r="C2" s="16" t="inlineStr">
+        <is>
+          <t>ERP ventas (sintético)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>DSO</t>
+        </is>
+      </c>
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>CxC / ventas diarias</t>
+        </is>
+      </c>
+      <c r="C3" s="16" t="inlineStr">
+        <is>
+          <t>Balance + PyG</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>DIO</t>
+        </is>
+      </c>
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>Inventarios / costo diario</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>Balance + PyG</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>DPO</t>
+        </is>
+      </c>
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>CxP / compras diarias</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="inlineStr">
+        <is>
+          <t>Balance + compras</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>DSO + DIO − DPO</t>
+        </is>
+      </c>
+      <c r="C6" s="16" t="inlineStr">
+        <is>
+          <t>Calculado</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Exposición USD</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>CxP USD − caja USD</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Tesorería</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Bridge EBITDA</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>Atribución volumen/precio/FX/descuento/opex</t>
+        </is>
+      </c>
+      <c r="C8" s="16" t="inlineStr">
+        <is>
+          <t>FP&amp;A</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Forecast base</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>Ventas 58.5M, EBITDA 5.4M, pico deuda oct 11.2M</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="inlineStr">
+        <is>
+          <t>Modelo + acciones A1-A5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>H1-2025</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Ventas 26.9M, EBITDA 2.76M: crece +5.6% YoY pero el margen se comprime</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Comparativo like-for-like</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Puente PVM</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>Volumen -1.10M, precio +250k, mix -450k, descuento -400k</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="inlineStr">
+        <is>
+          <t>FP&amp;A (ventas ppto-&gt;real)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Aging institucional</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>2.00M en 8 clientes, mora 60+ de 330k (DSO 70d del canal)</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>Auxiliar cobranza (sintetico)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>SKUs Hogar</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>3.35M en 8 SKUs, 3 con +6 meses de cobertura (702k)</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>Auxiliar inventarios (sintetico)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2420,165 +3438,286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Campo</t>
-        </is>
-      </c>
-      <c r="B1" s="10" t="inlineStr">
-        <is>
-          <t>Definición</t>
-        </is>
-      </c>
-      <c r="C1" s="10" t="inlineStr">
-        <is>
-          <t>Origen</t>
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Comparativo H1-2025 vs H1-2026 (S/) — like-for-like</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Cuenta</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>H1-2025</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>H1-2026 real</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Var YoY</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Var %</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Ventas netas</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
-        <is>
-          <t>Ventas brutas menos devoluciones y descuentos</t>
-        </is>
-      </c>
-      <c r="C2" s="16" t="inlineStr">
-        <is>
-          <t>ERP ventas (sintético)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>DSO</t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>CxC / ventas diarias</t>
-        </is>
-      </c>
-      <c r="C3" s="16" t="inlineStr">
-        <is>
-          <t>Balance + PyG</t>
-        </is>
+      <c r="B3" s="9" t="n">
+        <v>26900000</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>28400000</v>
+      </c>
+      <c r="D3" s="9">
+        <f>C3-B3</f>
+        <v/>
+      </c>
+      <c r="E3" s="8">
+        <f>IF(B3=0,0,C3/B3-1)</f>
+        <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
-        <is>
-          <t>DIO</t>
-        </is>
-      </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Inventarios / costo diario</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr">
-        <is>
-          <t>Balance + PyG</t>
-        </is>
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Costo de ventas</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>20659200</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>22123600</v>
+      </c>
+      <c r="D4" s="9">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="8">
+        <f>IF(B4=0,0,C4/B4-1)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>DPO</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>CxP / compras diarias</t>
-        </is>
-      </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>Balance + compras</t>
-        </is>
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Utilidad bruta</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>6240800</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>6276400</v>
+      </c>
+      <c r="D5" s="12">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>IF(B5=0,0,C5/B5-1)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
-        <is>
-          <t>CCC</t>
-        </is>
-      </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>DSO + DIO − DPO</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Calculado</t>
-        </is>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Gastos operativos</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>3480000</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>3926400</v>
+      </c>
+      <c r="D6" s="9">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
+        <f>IF(B6=0,0,C6/B6-1)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
-        <is>
-          <t>Exposición USD</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>CxP USD − caja USD</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>Tesorería</t>
-        </is>
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2760800</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>2350000</v>
+      </c>
+      <c r="D7" s="12">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="13">
+        <f>IF(B7=0,0,C7/B7-1)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
-        <is>
-          <t>Bridge EBITDA</t>
-        </is>
-      </c>
-      <c r="B8" s="16" t="inlineStr">
-        <is>
-          <t>Atribución volumen/precio/FX/descuento/opex</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>FP&amp;A</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Forecast base</t>
-        </is>
-      </c>
-      <c r="B9" s="16" t="inlineStr">
-        <is>
-          <t>Ventas 58.5M, EBITDA 5.4M, pico deuda oct 11.2M</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="inlineStr">
-        <is>
-          <t>Modelo + acciones A1-A5</t>
-        </is>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Utilidad neta</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>1192014</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>662700</v>
+      </c>
+      <c r="D8" s="12">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>IF(B8=0,0,C8/B8-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Por canal — ventas (S/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Canal</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>H1-2025</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>H1-2026 real</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Var YoY</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Ppto H1</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Vs ppto</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Mayorista</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>12600000</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>13314000</v>
+      </c>
+      <c r="D12" s="9">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>13545000</v>
+      </c>
+      <c r="F12" s="9">
+        <f>C12-E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Minorista</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>9400000</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>9942000</v>
+      </c>
+      <c r="D13" s="9">
+        <f>C13-B13</f>
+        <v/>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>10535000</v>
+      </c>
+      <c r="F13" s="9">
+        <f>C13-E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Institucional</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>5144000</v>
+      </c>
+      <c r="D14" s="9">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>6020000</v>
+      </c>
+      <c r="F14" s="9">
+        <f>C14-E14</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FP&A Pack V3: esquema Supabase fpa_*, demo en vivo con fallback y drill-down organico
</commit_message>
<xml_diff>
--- a/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
+++ b/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
@@ -1332,20 +1332,26 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>HOG-RESTO</t>
+          <t>HOG-VAR</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Resto linea Hogar (agregado)</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="12" t="n">
+          <t>Varios Hogar (agregado)</t>
+        </is>
+      </c>
+      <c r="C10" s="6" t="n">
+        <v>163620</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="9" t="n">
         <v>1636200</v>
       </c>
-      <c r="F10" s="6" t="n"/>
+      <c r="F10" s="6" t="n">
+        <v>77914</v>
+      </c>
       <c r="G10" s="15" t="n">
         <v>2.1</v>
       </c>

</xml_diff>

<commit_message>
FP&A Pack V4: waterfall reconciliado, flujo H1, supuestos LTM, factual fixes
</commit_message>
<xml_diff>
--- a/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
+++ b/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
@@ -14,12 +14,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BAL" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPIs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BRIDGE" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX_FORECAST" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMP_LY" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUENTE_VENTAS" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRILL_CLIENTES" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRILL_SKUS" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DICC" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FLUJO" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORECAST_H2" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FX_FORECAST" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="COMP_LY" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUENTE_VENTAS" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRILL_CLIENTES" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DRILL_SKUS" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DICC" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -499,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="130" customWidth="1" min="1" max="1"/>
@@ -564,47 +566,61 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>BRIDGE: puente EBITDA ppto → real (atribuye los -950k)</t>
+          <t>BRIDGE: puente EBITDA ppto → real reconciliado con el PVM (margen std 24%)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>COMP_LY: H1-2025 vs H1-2026 like-for-like + canales YoY</t>
+          <t>FLUJO: caja H1 indirecta que ata neta + WC + deuda = Δcaja -250k</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>PUENTE_VENTAS: volumen, precio, mix y descuento (atribuye los -1.70M)</t>
+          <t>FORECAST_H2: deuda mensual jul-dic con pico en octubre (supuesto base)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>DRILL_CLIENTES: CxC institucional por cliente y aging, con DSO</t>
+          <t>COMP_LY: H1-2025 vs H1-2026 like-for-like + canales YoY</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>DRILL_SKUS: inventarios Hogar por SKU, valorizado y cobertura</t>
+          <t>PUENTE_VENTAS: volumen, precio, mix y descuento (atribuye los -1.70M)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>FX_FORECAST: exposición USD, sensibilidad y forecast FY con plan de acción</t>
+          <t>DRILL_CLIENTES: CxC institucional por cliente y aging, con DSO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>DRILL_SKUS: inventarios Hogar por SKU, valorizado y cobertura</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>FX_FORECAST: exposición USD, sensibilidad y forecast FY con plan de acción</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>DICC: diccionario de campos y linaje</t>
         </is>
@@ -626,6 +642,636 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Exposición cambiaria (jun-26)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>CxP exterior (USD)</t>
+        </is>
+      </c>
+      <c r="B2" s="9" t="n">
+        <v>1350000</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Caja USD</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>-250000</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Exposición neta pasiva (USD)</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>1100000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Sensibilidad por 10 cts (PEN)</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>% sobre utilidad neta H1</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>16.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Forecast FY26 — escenario base con plan de acción</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Ppto FY</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Base FY</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Desvío</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Ventas</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>60200000</v>
+      </c>
+      <c r="C10" s="9" t="n">
+        <v>58500000</v>
+      </c>
+      <c r="D10" s="9">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>6700000</v>
+      </c>
+      <c r="C11" s="9" t="n">
+        <v>5400000</v>
+      </c>
+      <c r="D11" s="9">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Utilidad neta</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>3100000</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>1700000</v>
+      </c>
+      <c r="D12" s="9">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Pico deuda octubre (base)</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>11200000</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Línea adicional propuesta</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>2500000</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Plan de acción (efectos 2H)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Acción</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>Efecto caja</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>Efecto PyG</t>
+        </is>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>KPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Cobranza institucional + pronto pago</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="n">
+        <v>950000</v>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>- S/ 60k descuento financiero</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>DSO 52 -&gt; 46 dias</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Ajuste lista de precios 2H (+2%)</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>550000</v>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>+ S/ 550k margen</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr">
+        <is>
+          <t>Margen bruto +90 pbs en 2H</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Recorte compra hogar -15%</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="n">
+        <v>700000</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>neutro</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>DIO 61 -&gt; 55 dias</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Forward 50% exposicion 90 dias</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>acota riesgo 110k -&gt; 55k por 10 cts</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>Exposicion neta USD 1.10M -&gt; 0.55M</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>Linea revolvente +S/ 2.5M</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>- S/ 90k intereses 2H</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>Cubre pico de octubre</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Comparativo H1-2025 vs H1-2026 (S/) — like-for-like</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Cuenta</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>H1-2025</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>H1-2026 real</t>
+        </is>
+      </c>
+      <c r="D2" s="10" t="inlineStr">
+        <is>
+          <t>Var YoY</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Var %</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Ventas netas</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>26900000</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>28400000</v>
+      </c>
+      <c r="D3" s="9">
+        <f>C3-B3</f>
+        <v/>
+      </c>
+      <c r="E3" s="8">
+        <f>IF(B3=0,0,C3/B3-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Costo de ventas</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>20659200</v>
+      </c>
+      <c r="C4" s="9" t="n">
+        <v>22123600</v>
+      </c>
+      <c r="D4" s="9">
+        <f>C4-B4</f>
+        <v/>
+      </c>
+      <c r="E4" s="8">
+        <f>IF(B4=0,0,C4/B4-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>Utilidad bruta</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="n">
+        <v>6240800</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>6276400</v>
+      </c>
+      <c r="D5" s="12">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="13">
+        <f>IF(B5=0,0,C5/B5-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Gastos operativos</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n">
+        <v>3480000</v>
+      </c>
+      <c r="C6" s="9" t="n">
+        <v>3926400</v>
+      </c>
+      <c r="D6" s="9">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
+        <f>IF(B6=0,0,C6/B6-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="n">
+        <v>2760800</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>2350000</v>
+      </c>
+      <c r="D7" s="12">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="13">
+        <f>IF(B7=0,0,C7/B7-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Utilidad neta</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
+        <v>1192014</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>662700</v>
+      </c>
+      <c r="D8" s="12">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="13">
+        <f>IF(B8=0,0,C8/B8-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Por canal — ventas (S/)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Canal</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>H1-2025</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>H1-2026 real</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Var YoY</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Ppto H1</t>
+        </is>
+      </c>
+      <c r="F11" s="10" t="inlineStr">
+        <is>
+          <t>Vs ppto</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>Mayorista</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>12600000</v>
+      </c>
+      <c r="C12" s="9" t="n">
+        <v>13314000</v>
+      </c>
+      <c r="D12" s="9">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="9" t="n">
+        <v>13545000</v>
+      </c>
+      <c r="F12" s="9">
+        <f>C12-E12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Minorista</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>9400000</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>9942000</v>
+      </c>
+      <c r="D13" s="9">
+        <f>C13-B13</f>
+        <v/>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>10535000</v>
+      </c>
+      <c r="F13" s="9">
+        <f>C13-E13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Institucional</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>4900000</v>
+      </c>
+      <c r="C14" s="9" t="n">
+        <v>5144000</v>
+      </c>
+      <c r="D14" s="9">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="9" t="n">
+        <v>6020000</v>
+      </c>
+      <c r="F14" s="9">
+        <f>C14-E14</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -734,7 +1380,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1078,7 +1724,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1372,13 +2018,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1542,66 +2188,100 @@
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>H1-2025</t>
+          <t>Flujo H1</t>
         </is>
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Ventas 26.9M, EBITDA 2.76M: crece +5.6% YoY pero el margen se comprime</t>
+          <t>FCO -1.13M, capex -350k, deuda neta +1.23M, caja -250k</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Comparativo like-for-like</t>
+          <t>PyG + Balance</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Puente PVM</t>
+          <t>Deuda H2</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>Volumen -1.10M, precio +250k, mix -450k, descuento -400k</t>
+          <t>jul 10.4 a oct 11.2 y dic 10.0 (supuesto base)</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>FP&amp;A (ventas ppto-&gt;real)</t>
+          <t>Escenario, no ERP</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Aging institucional</t>
+          <t>H1-2025</t>
         </is>
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>2.00M en 8 clientes, mora 60+ de 330k (DSO 70d del canal)</t>
+          <t>Ventas 26.9M, EBITDA 2.76M: crece +5.6% YoY pero el margen se comprime</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>Auxiliar cobranza (sintetico)</t>
+          <t>Comparativo like-for-like</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
+          <t>Puente PVM</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>Volumen -1.10M, precio +250k, mix -450k, descuento -400k</t>
+        </is>
+      </c>
+      <c r="C13" s="16" t="inlineStr">
+        <is>
+          <t>FP&amp;A (ventas ppto-&gt;real)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Aging institucional</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>2.00M en 8 clientes, mora 60+ de 330k (DSO 70d del canal)</t>
+        </is>
+      </c>
+      <c r="C14" s="16" t="inlineStr">
+        <is>
+          <t>Auxiliar cobranza (sintetico)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
           <t>SKUs Hogar</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>3.35M en 8 SKUs, 3 con +6 meses de cobertura (702k)</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>Auxiliar inventarios (sintetico)</t>
         </is>
@@ -2967,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3008,91 +3688,78 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Efecto volumen</t>
+          <t>Efecto volumen (margen std 24%)</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>-410000</v>
+        <v>-264000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>2890000</v>
+        <v>3036000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Efecto precio / mix</t>
+          <t>Efecto precio / mix / descuento</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>-120000</v>
+        <v>-144000</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>2770000</v>
+        <v>2892000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Efecto costo FX (TC 3.72-&gt;3.81)</t>
+          <t>Costo FX (TC 3.72-&gt;3.81)</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
         <v>-300000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>2470000</v>
+        <v>2592000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Descuento comercial defensivo</t>
+          <t>Otros costos</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>-120000</v>
+        <v>-239600</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2350000</v>
+        <v>2352400</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Fletes y personal</t>
+          <t>Opex neto</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>-180000</v>
+        <v>-2400</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2170000</v>
+        <v>2350000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>Ahorro marketing y variables</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>180000</v>
-      </c>
-      <c r="C8" s="9" t="n">
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>EBITDA real H1</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="n">
         <v>2350000</v>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>EBITDA real H1</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="n">
-        <v>2350000</v>
-      </c>
-      <c r="C9" s="12" t="n">
+      <c r="C8" s="12" t="n">
         <v>2350000</v>
       </c>
     </row>
@@ -3107,330 +3774,185 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Exposición cambiaria (jun-26)</t>
+          <t>Flujo de caja H1 indirecto (S/) — ata Δcaja -250k</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>CxP exterior (USD)</t>
-        </is>
-      </c>
-      <c r="B2" s="9" t="n">
-        <v>1350000</v>
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B2" s="10" t="inlineStr">
+        <is>
+          <t>Monto</t>
+        </is>
+      </c>
+      <c r="C2" s="10" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Caja USD</t>
+          <t>Utilidad neta</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>-250000</v>
-      </c>
+        <v>662700</v>
+      </c>
+      <c r="C3" s="6" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Exposición neta pasiva (USD)</t>
+          <t>Depreciación</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1100000</v>
-      </c>
+        <v>450000</v>
+      </c>
+      <c r="C4" s="6" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Sensibilidad por 10 cts (PEN)</t>
+          <t>Δ Cuentas por cobrar</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>110000</v>
-      </c>
+        <v>-1360000</v>
+      </c>
+      <c r="C5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>% sobre utilidad neta H1</t>
+          <t>Δ Inventarios</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>16.6</v>
-      </c>
+        <v>-800000</v>
+      </c>
+      <c r="C6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Δ Cuentas por pagar comerciales</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>-180000</v>
+      </c>
+      <c r="C7" s="6" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Forecast FY26 — escenario base con plan de acción</t>
-        </is>
-      </c>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Δ Otros pasivos CP</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>100000</v>
+      </c>
+      <c r="C8" s="6" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="10" t="inlineStr">
-        <is>
-          <t>Concepto</t>
-        </is>
-      </c>
-      <c r="B9" s="10" t="inlineStr">
-        <is>
-          <t>Ppto FY</t>
-        </is>
-      </c>
-      <c r="C9" s="10" t="inlineStr">
-        <is>
-          <t>Base FY</t>
-        </is>
-      </c>
-      <c r="D9" s="10" t="inlineStr">
-        <is>
-          <t>Desvío</t>
-        </is>
+      <c r="A9" s="11" t="inlineStr">
+        <is>
+          <t>FLUJO OPERATIVO</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="n">
+        <v>-1127300</v>
+      </c>
+      <c r="C9" s="6">
+        <f>SUM(B3:B8)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Capex</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>60200000</v>
-      </c>
-      <c r="C10" s="9" t="n">
-        <v>58500000</v>
-      </c>
-      <c r="D10" s="9">
-        <f>C10-B10</f>
-        <v/>
-      </c>
+        <v>-350000</v>
+      </c>
+      <c r="C10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>EBITDA</t>
+          <t>Δ Deuda CP</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>6700000</v>
-      </c>
-      <c r="C11" s="9" t="n">
-        <v>5400000</v>
-      </c>
-      <c r="D11" s="9">
-        <f>C11-B11</f>
-        <v/>
-      </c>
+        <v>2297300</v>
+      </c>
+      <c r="C11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Utilidad neta</t>
+          <t>Δ Deuda LP</t>
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>3100000</v>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>1700000</v>
-      </c>
-      <c r="D12" s="9">
-        <f>C12-B12</f>
-        <v/>
-      </c>
+        <v>-1070000</v>
+      </c>
+      <c r="C12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Pico deuda octubre (base)</t>
+          <t>Δ CAJA (dic-&gt;jun)</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>11200000</v>
+        <v>-250000</v>
+      </c>
+      <c r="C13" s="6">
+        <f>B9+B10+B11+B12+B13</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Línea adicional propuesta</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>2500000</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Plan de acción (efectos 2H)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="inlineStr">
-        <is>
-          <t>Acción</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Efecto caja</t>
-        </is>
-      </c>
-      <c r="D17" s="10" t="inlineStr">
-        <is>
-          <t>Efecto PyG</t>
-        </is>
-      </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>KPI</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Cobranza institucional + pronto pago</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="n">
-        <v>950000</v>
-      </c>
-      <c r="D18" s="4" t="inlineStr">
-        <is>
-          <t>- S/ 60k descuento financiero</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="inlineStr">
-        <is>
-          <t>DSO 52 -&gt; 46 dias</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Ajuste lista de precios 2H (+2%)</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="n">
-        <v>550000</v>
-      </c>
-      <c r="D19" s="4" t="inlineStr">
-        <is>
-          <t>+ S/ 550k margen</t>
-        </is>
-      </c>
-      <c r="E19" s="4" t="inlineStr">
-        <is>
-          <t>Margen bruto +90 pbs en 2H</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>A3</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Recorte compra hogar -15%</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="n">
-        <v>700000</v>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>neutro</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>DIO 61 -&gt; 55 dias</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>A4</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Forward 50% exposicion 90 dias</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>acota riesgo 110k -&gt; 55k por 10 cts</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="inlineStr">
-        <is>
-          <t>Exposicion neta USD 1.10M -&gt; 0.55M</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Linea revolvente +S/ 2.5M</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="n">
-        <v>2500000</v>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>- S/ 90k intereses 2H</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr">
-        <is>
-          <t>Cubre pico de octubre</t>
-        </is>
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t>Check FCO (debe dar 0)</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Check caja (debe dar 0)</t>
+        </is>
+      </c>
+      <c r="B15" s="12">
+        <f>C13-B13</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -3444,286 +3966,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Comparativo H1-2025 vs H1-2026 (S/) — like-for-like</t>
+          <t>Deuda total fin de mes jul-dic 2026 base (S/) — supuesto, pico octubre</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Cuenta</t>
+          <t>Mes</t>
         </is>
       </c>
       <c r="B2" s="10" t="inlineStr">
         <is>
-          <t>H1-2025</t>
-        </is>
-      </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>H1-2026 real</t>
-        </is>
-      </c>
-      <c r="D2" s="10" t="inlineStr">
-        <is>
-          <t>Var YoY</t>
-        </is>
-      </c>
-      <c r="E2" s="10" t="inlineStr">
-        <is>
-          <t>Var %</t>
+          <t>Deuda fin de mes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Ventas netas</t>
+          <t>Jul</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>26900000</v>
-      </c>
-      <c r="C3" s="9" t="n">
-        <v>28400000</v>
-      </c>
-      <c r="D3" s="9">
-        <f>C3-B3</f>
-        <v/>
-      </c>
-      <c r="E3" s="8">
-        <f>IF(B3=0,0,C3/B3-1)</f>
-        <v/>
+        <v>10400000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Costo de ventas</t>
+          <t>Ago</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>20659200</v>
-      </c>
-      <c r="C4" s="9" t="n">
-        <v>22123600</v>
-      </c>
-      <c r="D4" s="9">
-        <f>C4-B4</f>
-        <v/>
-      </c>
-      <c r="E4" s="8">
-        <f>IF(B4=0,0,C4/B4-1)</f>
-        <v/>
+        <v>10700000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
-        <is>
-          <t>Utilidad bruta</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="n">
-        <v>6240800</v>
-      </c>
-      <c r="C5" s="12" t="n">
-        <v>6276400</v>
-      </c>
-      <c r="D5" s="12">
-        <f>C5-B5</f>
-        <v/>
-      </c>
-      <c r="E5" s="13">
-        <f>IF(B5=0,0,C5/B5-1)</f>
-        <v/>
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Sep</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>10900000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Gastos operativos</t>
-        </is>
-      </c>
-      <c r="B6" s="9" t="n">
-        <v>3480000</v>
-      </c>
-      <c r="C6" s="9" t="n">
-        <v>3926400</v>
-      </c>
-      <c r="D6" s="9">
-        <f>C6-B6</f>
-        <v/>
-      </c>
-      <c r="E6" s="8">
-        <f>IF(B6=0,0,C6/B6-1)</f>
-        <v/>
+          <t>Oct</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="n">
+        <v>11200000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
-        <is>
-          <t>EBITDA</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="n">
-        <v>2760800</v>
-      </c>
-      <c r="C7" s="12" t="n">
-        <v>2350000</v>
-      </c>
-      <c r="D7" s="12">
-        <f>C7-B7</f>
-        <v/>
-      </c>
-      <c r="E7" s="13">
-        <f>IF(B7=0,0,C7/B7-1)</f>
-        <v/>
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Nov</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>10600000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
-        <is>
-          <t>Utilidad neta</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="n">
-        <v>1192014</v>
-      </c>
-      <c r="C8" s="12" t="n">
-        <v>662700</v>
-      </c>
-      <c r="D8" s="12">
-        <f>C8-B8</f>
-        <v/>
-      </c>
-      <c r="E8" s="13">
-        <f>IF(B8=0,0,C8/B8-1)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Por canal — ventas (S/)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Canal</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="inlineStr">
-        <is>
-          <t>H1-2025</t>
-        </is>
-      </c>
-      <c r="C11" s="10" t="inlineStr">
-        <is>
-          <t>H1-2026 real</t>
-        </is>
-      </c>
-      <c r="D11" s="10" t="inlineStr">
-        <is>
-          <t>Var YoY</t>
-        </is>
-      </c>
-      <c r="E11" s="10" t="inlineStr">
-        <is>
-          <t>Ppto H1</t>
-        </is>
-      </c>
-      <c r="F11" s="10" t="inlineStr">
-        <is>
-          <t>Vs ppto</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Mayorista</t>
-        </is>
-      </c>
-      <c r="B12" s="9" t="n">
-        <v>12600000</v>
-      </c>
-      <c r="C12" s="9" t="n">
-        <v>13314000</v>
-      </c>
-      <c r="D12" s="9">
-        <f>C12-B12</f>
-        <v/>
-      </c>
-      <c r="E12" s="9" t="n">
-        <v>13545000</v>
-      </c>
-      <c r="F12" s="9">
-        <f>C12-E12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Minorista</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="n">
-        <v>9400000</v>
-      </c>
-      <c r="C13" s="9" t="n">
-        <v>9942000</v>
-      </c>
-      <c r="D13" s="9">
-        <f>C13-B13</f>
-        <v/>
-      </c>
-      <c r="E13" s="9" t="n">
-        <v>10535000</v>
-      </c>
-      <c r="F13" s="9">
-        <f>C13-E13</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Institucional</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="n">
-        <v>4900000</v>
-      </c>
-      <c r="C14" s="9" t="n">
-        <v>5144000</v>
-      </c>
-      <c r="D14" s="9">
-        <f>C14-B14</f>
-        <v/>
-      </c>
-      <c r="E14" s="9" t="n">
-        <v>6020000</v>
-      </c>
-      <c r="F14" s="9">
-        <f>C14-E14</f>
-        <v/>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Dic</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>10000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
FPA V5: caso nuevo Comercial Los Alamos (escala/sector distintos), seed DO UPDATE
</commit_message>
<xml_diff>
--- a/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
+++ b/assets/demo/fpa-pack/fpa_pack_jun2026.xlsx
@@ -510,7 +510,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Distribuidora Andina del Sur S.A.C.</t>
+          <t>Comercial Los Alamos S.A.C.</t>
         </is>
       </c>
     </row>
@@ -594,21 +594,21 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>PUENTE_VENTAS: volumen, precio, mix y descuento (atribuye los -1.70M)</t>
+          <t>PUENTE_VENTAS: volumen, precio, mix y descuento (atribuye el desvio de ventas)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>DRILL_CLIENTES: CxC institucional por cliente y aging, con DSO</t>
+          <t>DRILL_CLIENTES: CxC Constructor por cliente y aging, con DSO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>DRILL_SKUS: inventarios Hogar por SKU, valorizado y cobertura</t>
+          <t>DRILL_SKUS: inventarios Acabados por SKU, valorizado y cobertura</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>1350000</v>
+        <v>220000</v>
       </c>
     </row>
     <row r="3">
@@ -676,7 +676,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>-250000</v>
+        <v>-40000</v>
       </c>
     </row>
     <row r="4">
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>1100000</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="5">
@@ -696,7 +696,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>110000</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="6">
@@ -706,7 +706,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>16.6</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="8">
@@ -745,10 +745,10 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>60200000</v>
+        <v>24000000</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>58500000</v>
+        <v>23100000</v>
       </c>
       <c r="D10" s="9">
         <f>C10-B10</f>
@@ -762,10 +762,10 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>6700000</v>
+        <v>2880000</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>5400000</v>
+        <v>2250000</v>
       </c>
       <c r="D11" s="9">
         <f>C11-B11</f>
@@ -779,10 +779,10 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>3100000</v>
+        <v>1410000</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>1700000</v>
+        <v>720000</v>
       </c>
       <c r="D12" s="9">
         <f>C12-B12</f>
@@ -796,7 +796,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>11200000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="14">
@@ -806,7 +806,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>2500000</v>
+        <v>1000000</v>
       </c>
     </row>
     <row r="16">
@@ -851,15 +851,15 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Cobranza institucional + pronto pago</t>
+          <t>Cobranza constructor + pronto pago</t>
         </is>
       </c>
       <c r="C18" s="9" t="n">
-        <v>950000</v>
+        <v>375000</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>- S/ 60k descuento financiero</t>
+          <t>- S/ 25k descuento financiero</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -880,16 +880,16 @@
         </is>
       </c>
       <c r="C19" s="9" t="n">
-        <v>550000</v>
+        <v>220000</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>+ S/ 550k margen</t>
+          <t>+ S/ 220k margen</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>Margen bruto +90 pbs en 2H</t>
+          <t>Margen bruto +80 pbs en 2H</t>
         </is>
       </c>
     </row>
@@ -901,11 +901,11 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>Recorte compra hogar -15%</t>
+          <t>Recorte compra acabados -15%</t>
         </is>
       </c>
       <c r="C20" s="9" t="n">
-        <v>700000</v>
+        <v>280000</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
@@ -934,12 +934,12 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>acota riesgo 110k -&gt; 55k por 10 cts</t>
+          <t>acota riesgo 18k -&gt; 9k por 10 cts</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Exposicion neta USD 1.10M -&gt; 0.55M</t>
+          <t>Exposicion neta USD 180k -&gt; 90k</t>
         </is>
       </c>
     </row>
@@ -951,15 +951,15 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Linea revolvente +S/ 2.5M</t>
+          <t>Linea revolvente +S/ 1.0M</t>
         </is>
       </c>
       <c r="C22" s="9" t="n">
-        <v>2500000</v>
+        <v>1000000</v>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>- S/ 90k intereses 2H</t>
+          <t>- S/ 35k intereses 2H</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
@@ -1031,10 +1031,10 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>26900000</v>
+        <v>10700000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>28400000</v>
+        <v>11300000</v>
       </c>
       <c r="D3" s="9">
         <f>C3-B3</f>
@@ -1052,10 +1052,10 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>20659200</v>
+        <v>8014300</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>22123600</v>
+        <v>8565400</v>
       </c>
       <c r="D4" s="9">
         <f>C4-B4</f>
@@ -1073,10 +1073,10 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>6240800</v>
+        <v>2685700</v>
       </c>
       <c r="C5" s="12" t="n">
-        <v>6276400</v>
+        <v>2734600</v>
       </c>
       <c r="D5" s="12">
         <f>C5-B5</f>
@@ -1094,10 +1094,10 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>3480000</v>
+        <v>1450000</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>3926400</v>
+        <v>1684600</v>
       </c>
       <c r="D6" s="9">
         <f>C6-B6</f>
@@ -1115,10 +1115,10 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>2760800</v>
+        <v>1235700</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>2350000</v>
+        <v>1050000</v>
       </c>
       <c r="D7" s="12">
         <f>C7-B7</f>
@@ -1136,10 +1136,10 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>1192014</v>
+        <v>568018</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>662700</v>
+        <v>341925</v>
       </c>
       <c r="D8" s="12">
         <f>C8-B8</f>
@@ -1192,21 +1192,21 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Mayorista</t>
+          <t>Ferretero</t>
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>12600000</v>
+        <v>5000000</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>13314000</v>
+        <v>5130000</v>
       </c>
       <c r="D12" s="9">
         <f>C12-B12</f>
         <v/>
       </c>
       <c r="E12" s="9" t="n">
-        <v>13545000</v>
+        <v>5400000</v>
       </c>
       <c r="F12" s="9">
         <f>C12-E12</f>
@@ -1216,21 +1216,21 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Minorista</t>
+          <t>Constructor</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>9400000</v>
+        <v>3600000</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>9942000</v>
+        <v>3840000</v>
       </c>
       <c r="D13" s="9">
         <f>C13-B13</f>
         <v/>
       </c>
       <c r="E13" s="9" t="n">
-        <v>10535000</v>
+        <v>4200000</v>
       </c>
       <c r="F13" s="9">
         <f>C13-E13</f>
@@ -1240,21 +1240,21 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Institucional</t>
+          <t>Retail</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>4900000</v>
+        <v>2100000</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>5144000</v>
+        <v>2330000</v>
       </c>
       <c r="D14" s="9">
         <f>C14-B14</f>
         <v/>
       </c>
       <c r="E14" s="9" t="n">
-        <v>6020000</v>
+        <v>2400000</v>
       </c>
       <c r="F14" s="9">
         <f>C14-E14</f>
@@ -1304,10 +1304,10 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>30100000</v>
+        <v>12000000</v>
       </c>
       <c r="C2" s="12" t="n">
-        <v>30100000</v>
+        <v>12000000</v>
       </c>
     </row>
     <row r="3">
@@ -1317,10 +1317,10 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>-1100000</v>
+        <v>-450000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>29000000</v>
+        <v>11550000</v>
       </c>
     </row>
     <row r="4">
@@ -1330,10 +1330,10 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>250000</v>
+        <v>110000</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>29250000</v>
+        <v>11660000</v>
       </c>
     </row>
     <row r="5">
@@ -1343,10 +1343,10 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>-450000</v>
+        <v>-180000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>28800000</v>
+        <v>11480000</v>
       </c>
     </row>
     <row r="6">
@@ -1356,10 +1356,10 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>-400000</v>
+        <v>-180000</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>28400000</v>
+        <v>11300000</v>
       </c>
     </row>
     <row r="7">
@@ -1369,10 +1369,10 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>28400000</v>
+        <v>11300000</v>
       </c>
       <c r="C7" s="12" t="n">
-        <v>28400000</v>
+        <v>11300000</v>
       </c>
     </row>
   </sheetData>
@@ -1402,7 +1402,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Drill-down cobranza — CxC Institucional S/ 2.00M por cliente y aging (S/)</t>
+          <t>Drill-down cobranza — CxC Constructor S/ 0,80M por cliente y aging (S/)</t>
         </is>
       </c>
     </row>
@@ -1455,13 +1455,13 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>300000</v>
+        <v>120000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>150000</v>
+        <v>60000</v>
       </c>
       <c r="D3" s="9" t="n">
-        <v>70000</v>
+        <v>28000</v>
       </c>
       <c r="E3" s="9" t="n">
         <v>0</v>
@@ -1471,7 +1471,7 @@
         <v/>
       </c>
       <c r="G3" s="15" t="n">
-        <v>18.3</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="H3" s="9">
         <f>D3+E3</f>
@@ -1485,23 +1485,23 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>200000</v>
+        <v>80000</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>120000</v>
+        <v>48000</v>
       </c>
       <c r="D4" s="9" t="n">
-        <v>60000</v>
+        <v>24000</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="F4" s="12">
         <f>SUM(B4:E4)</f>
         <v/>
       </c>
       <c r="G4" s="15" t="n">
-        <v>14.4</v>
+        <v>7.7</v>
       </c>
       <c r="H4" s="9">
         <f>D4+E4</f>
@@ -1515,13 +1515,13 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>250000</v>
+        <v>100000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>80000</v>
+        <v>32000</v>
       </c>
       <c r="D5" s="9" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="E5" s="9" t="n">
         <v>0</v>
@@ -1531,7 +1531,7 @@
         <v/>
       </c>
       <c r="G5" s="15" t="n">
-        <v>12.3</v>
+        <v>6.6</v>
       </c>
       <c r="H5" s="9">
         <f>D5+E5</f>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>280000</v>
+        <v>112000</v>
       </c>
       <c r="C6" s="9" t="n">
         <v>0</v>
@@ -1561,7 +1561,7 @@
         <v/>
       </c>
       <c r="G6" s="15" t="n">
-        <v>9.9</v>
+        <v>5.3</v>
       </c>
       <c r="H6" s="9">
         <f>D6+E6</f>
@@ -1575,13 +1575,13 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>50000</v>
+        <v>20000</v>
       </c>
       <c r="D7" s="9" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="E7" s="9" t="n">
         <v>0</v>
@@ -1591,7 +1591,7 @@
         <v/>
       </c>
       <c r="G7" s="15" t="n">
-        <v>6.3</v>
+        <v>3.4</v>
       </c>
       <c r="H7" s="9">
         <f>D7+E7</f>
@@ -1605,23 +1605,23 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>40000</v>
+        <v>16000</v>
       </c>
       <c r="C8" s="9" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="D8" s="9" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="F8" s="12">
         <f>SUM(B8:E8)</f>
         <v/>
       </c>
       <c r="G8" s="15" t="n">
-        <v>4.2</v>
+        <v>2.3</v>
       </c>
       <c r="H8" s="9">
         <f>D8+E8</f>
@@ -1638,20 +1638,20 @@
         <v>0</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="D9" s="9" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>40000</v>
+        <v>16000</v>
       </c>
       <c r="F9" s="12">
         <f>SUM(B9:E9)</f>
         <v/>
       </c>
       <c r="G9" s="15" t="n">
-        <v>3.2</v>
+        <v>1.7</v>
       </c>
       <c r="H9" s="9">
         <f>D9+E9</f>
@@ -1665,10 +1665,10 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>30000</v>
+        <v>12000</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>20000</v>
+        <v>8000</v>
       </c>
       <c r="D10" s="9" t="n">
         <v>0</v>
@@ -1681,7 +1681,7 @@
         <v/>
       </c>
       <c r="G10" s="15" t="n">
-        <v>1.8</v>
+        <v>0.9</v>
       </c>
       <c r="H10" s="9">
         <f>D10+E10</f>
@@ -1745,7 +1745,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Drill-down inventarios — linea Hogar S/ 3.35M por SKU</t>
+          <t>Drill-down inventarios — linea Acabados S/ 1,39M por SKU</t>
         </is>
       </c>
     </row>
@@ -1789,25 +1789,25 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>HOG-014</t>
+          <t>CER-101</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>Detergente industrial 20kg</t>
+          <t>Porcelanato 60x60 caja</t>
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>14000</v>
+        <v>2100</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>18.5</v>
+        <v>68</v>
       </c>
       <c r="E3" s="9" t="n">
-        <v>259000</v>
+        <v>142800</v>
       </c>
       <c r="F3" s="6" t="n">
-        <v>3200</v>
+        <v>475</v>
       </c>
       <c r="G3" s="15" t="n">
         <v>4.4</v>
@@ -1816,79 +1816,79 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>HOG-022</t>
+          <t>PIN-020</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Jabon liquido 5L</t>
+          <t>Pintura latex 20L</t>
         </is>
       </c>
       <c r="C4" s="6" t="n">
-        <v>22000</v>
+        <v>1900</v>
       </c>
       <c r="D4" s="6" t="n">
-        <v>12.8</v>
+        <v>92.5</v>
       </c>
       <c r="E4" s="9" t="n">
-        <v>281600</v>
+        <v>175750</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>4800</v>
+        <v>390</v>
       </c>
       <c r="G4" s="15" t="n">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HOG-031</t>
+          <t>PEG-025</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Papel toalla x12</t>
+          <t>Pegamento ceramico 25kg</t>
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>30000</v>
+        <v>4500</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>9.4</v>
+        <v>24.8</v>
       </c>
       <c r="E5" s="9" t="n">
-        <v>282000</v>
+        <v>111600</v>
       </c>
       <c r="F5" s="6" t="n">
-        <v>7500</v>
+        <v>1100</v>
       </c>
       <c r="G5" s="15" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>HOG-007</t>
+          <t>LAC-011</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Desinfectante 1L</t>
+          <t>Laca selladora 1L</t>
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>45000</v>
+        <v>3250</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>4.2</v>
+        <v>18.9</v>
       </c>
       <c r="E6" s="9" t="n">
-        <v>189000</v>
+        <v>61425</v>
       </c>
       <c r="F6" s="6" t="n">
-        <v>12000</v>
+        <v>850</v>
       </c>
       <c r="G6" s="15" t="n">
         <v>3.8</v>
@@ -1897,25 +1897,25 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>HOG-045</t>
+          <t>PER-008</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Escobas premium</t>
+          <t>Perfiles aluminio 6m</t>
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>18000</v>
+        <v>1200</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>6.9</v>
+        <v>45</v>
       </c>
       <c r="E7" s="9" t="n">
-        <v>124200</v>
+        <v>54000</v>
       </c>
       <c r="F7" s="6" t="n">
-        <v>2100</v>
+        <v>140</v>
       </c>
       <c r="G7" s="15" t="n">
         <v>8.6</v>
@@ -1924,25 +1924,25 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>HOG-046</t>
+          <t>SAN-031</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Trapeadores</t>
+          <t>Griferia cocina</t>
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>25000</v>
+        <v>950</v>
       </c>
       <c r="D8" s="6" t="n">
-        <v>5.6</v>
+        <v>62</v>
       </c>
       <c r="E8" s="9" t="n">
-        <v>140000</v>
+        <v>58900</v>
       </c>
       <c r="F8" s="6" t="n">
-        <v>3000</v>
+        <v>115</v>
       </c>
       <c r="G8" s="15" t="n">
         <v>8.300000000000001</v>
@@ -1951,52 +1951,52 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>HOG-052</t>
+          <t>ILU-044</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Bolsas basura 100L x50</t>
+          <t>Focos LED 12W caja x24</t>
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>60000</v>
+        <v>2500</v>
       </c>
       <c r="D9" s="6" t="n">
-        <v>7.3</v>
+        <v>38.4</v>
       </c>
       <c r="E9" s="9" t="n">
-        <v>438000</v>
+        <v>96000</v>
       </c>
       <c r="F9" s="6" t="n">
-        <v>9000</v>
+        <v>360</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>6.7</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>HOG-VAR</t>
+          <t>ACA-VAR</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Varios Hogar (agregado)</t>
+          <t>Varios Acabados (agregado)</t>
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>163620</v>
+        <v>68642</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>10</v>
       </c>
       <c r="E10" s="9" t="n">
-        <v>1636200</v>
+        <v>686420</v>
       </c>
       <c r="F10" s="6" t="n">
-        <v>77914</v>
+        <v>32687</v>
       </c>
       <c r="G10" s="15" t="n">
         <v>2.1</v>
@@ -2176,7 +2176,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>Ventas 58.5M, EBITDA 5.4M, pico deuda oct 11.2M</t>
+          <t>Ventas S/ 23,10M, EBITDA S/ 2,25M, pico deuda oct S/ 4,50M</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
@@ -2256,12 +2256,12 @@
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
         <is>
-          <t>Aging institucional</t>
+          <t>Aging constructor</t>
         </is>
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>2.00M en 8 clientes, mora 60+ de 330k (DSO 70d del canal)</t>
+          <t>S/ 0,80M en 8 clientes, mora 60+ de S/ 132k (DSO 52d del canal)</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
@@ -2273,12 +2273,12 @@
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>SKUs Hogar</t>
+          <t>SKUs Acabados</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>3.35M en 8 SKUs, 3 con +6 meses de cobertura (702k)</t>
+          <t>S/ 1,39M en 8 SKUs, 3 con +6 meses de cobertura (S/ 209k)</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
@@ -2452,7 +2452,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>60200000</v>
+        <v>24000000</v>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
@@ -2467,7 +2467,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>2500000</v>
+        <v>1000000</v>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
@@ -2530,10 +2530,10 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>4600000</v>
+        <v>1800000</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>4550000</v>
+        <v>1760000</v>
       </c>
       <c r="D2" s="9">
         <f>C2-B2</f>
@@ -2551,10 +2551,10 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>4400000</v>
+        <v>1750000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>4200000</v>
+        <v>1680000</v>
       </c>
       <c r="D3" s="9">
         <f>C3-B3</f>
@@ -2572,10 +2572,10 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>5000000</v>
+        <v>2000000</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>4750000</v>
+        <v>1900000</v>
       </c>
       <c r="D4" s="9">
         <f>C4-B4</f>
@@ -2593,10 +2593,10 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>5000000</v>
+        <v>2000000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>4700000</v>
+        <v>1880000</v>
       </c>
       <c r="D5" s="9">
         <f>C5-B5</f>
@@ -2614,10 +2614,10 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>5200000</v>
+        <v>2100000</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>4850000</v>
+        <v>1950000</v>
       </c>
       <c r="D6" s="9">
         <f>C6-B6</f>
@@ -2635,10 +2635,10 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>5900000</v>
+        <v>2350000</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>5350000</v>
+        <v>2130000</v>
       </c>
       <c r="D7" s="9">
         <f>C7-B7</f>
@@ -2733,10 +2733,10 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>30100000</v>
+        <v>12000000</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>28400000</v>
+        <v>11300000</v>
       </c>
       <c r="D2" s="9">
         <f>C2-B2</f>
@@ -2759,10 +2759,10 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>22876000</v>
+        <v>8880000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>22123600</v>
+        <v>8565400</v>
       </c>
       <c r="D3" s="9">
         <f>C3-B3</f>
@@ -2785,10 +2785,10 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>7224000</v>
+        <v>3120000</v>
       </c>
       <c r="C4" s="12" t="n">
-        <v>6276400</v>
+        <v>2734600</v>
       </c>
       <c r="D4" s="12">
         <f>C4-B4</f>
@@ -2810,10 +2810,10 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>3924000</v>
+        <v>1680000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>3926400</v>
+        <v>1684600</v>
       </c>
       <c r="D5" s="9">
         <f>C5-B5</f>
@@ -2836,10 +2836,10 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>3300000</v>
+        <v>1440000</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>2350000</v>
+        <v>1050000</v>
       </c>
       <c r="D6" s="12">
         <f>C6-B6</f>
@@ -2887,10 +2887,10 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>2850000</v>
+        <v>1260000</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>1900000</v>
+        <v>870000</v>
       </c>
       <c r="D8" s="12">
         <f>C8-B8</f>
@@ -2912,10 +2912,10 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>550000</v>
+        <v>220000</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>680000</v>
+        <v>275000</v>
       </c>
       <c r="D9" s="9">
         <f>C9-B9</f>
@@ -2938,10 +2938,10 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>-100000</v>
+        <v>-40000</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>-280000</v>
+        <v>-110000</v>
       </c>
       <c r="D10" s="9">
         <f>C10-B10</f>
@@ -2964,10 +2964,10 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>2200000</v>
+        <v>1000000</v>
       </c>
       <c r="C11" s="12" t="n">
-        <v>940000</v>
+        <v>485000</v>
       </c>
       <c r="D11" s="12">
         <f>C11-B11</f>
@@ -2989,10 +2989,10 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>649000</v>
+        <v>295000</v>
       </c>
       <c r="C12" s="9" t="n">
-        <v>277300</v>
+        <v>143075</v>
       </c>
       <c r="D12" s="9">
         <f>C12-B12</f>
@@ -3015,10 +3015,10 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>1551000</v>
+        <v>705000</v>
       </c>
       <c r="C13" s="12" t="n">
-        <v>662700</v>
+        <v>341925</v>
       </c>
       <c r="D13" s="12">
         <f>C13-B13</f>
@@ -3088,10 +3088,10 @@
         </is>
       </c>
       <c r="B2" s="9" t="n">
-        <v>1200000</v>
+        <v>480000</v>
       </c>
       <c r="C2" s="9" t="n">
-        <v>950000</v>
+        <v>380000</v>
       </c>
       <c r="D2" s="9">
         <f>C2-B2</f>
@@ -3109,10 +3109,10 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>6800000</v>
+        <v>2720000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>8160000</v>
+        <v>3246400</v>
       </c>
       <c r="D3" s="9">
         <f>C3-B3</f>
@@ -3130,10 +3130,10 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>6650000</v>
+        <v>2660000</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>7450000</v>
+        <v>2886895</v>
       </c>
       <c r="D4" s="9">
         <f>C4-B4</f>
@@ -3151,10 +3151,10 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>400000</v>
+        <v>160000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>400000</v>
+        <v>160000</v>
       </c>
       <c r="D5" s="9">
         <f>C5-B5</f>
@@ -3172,10 +3172,10 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>15050000</v>
+        <v>6020000</v>
       </c>
       <c r="C6" s="12" t="n">
-        <v>16960000</v>
+        <v>6673295</v>
       </c>
       <c r="D6" s="12">
         <f>C6-B6</f>
@@ -3193,10 +3193,10 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>8450000</v>
+        <v>3380000</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>8350000</v>
+        <v>3370000</v>
       </c>
       <c r="D7" s="9">
         <f>C7-B7</f>
@@ -3214,10 +3214,10 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>23500000</v>
+        <v>9400000</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>25310000</v>
+        <v>10043295</v>
       </c>
       <c r="D8" s="12">
         <f>C8-B8</f>
@@ -3235,10 +3235,10 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>4500000</v>
+        <v>1800000</v>
       </c>
       <c r="C9" s="9" t="n">
-        <v>4320000</v>
+        <v>1651700</v>
       </c>
       <c r="D9" s="9">
         <f>C9-B9</f>
@@ -3256,10 +3256,10 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>3800000</v>
+        <v>1520000</v>
       </c>
       <c r="C10" s="9" t="n">
-        <v>6097300</v>
+        <v>2359670</v>
       </c>
       <c r="D10" s="9">
         <f>C10-B10</f>
@@ -3277,10 +3277,10 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>1000000</v>
+        <v>400000</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>1100000</v>
+        <v>440000</v>
       </c>
       <c r="D11" s="9">
         <f>C11-B11</f>
@@ -3298,10 +3298,10 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>9300000</v>
+        <v>3720000</v>
       </c>
       <c r="C12" s="12" t="n">
-        <v>11517300</v>
+        <v>4451370</v>
       </c>
       <c r="D12" s="12">
         <f>C12-B12</f>
@@ -3319,10 +3319,10 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>4970000</v>
+        <v>1990000</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>3900000</v>
+        <v>1560000</v>
       </c>
       <c r="D13" s="9">
         <f>C13-B13</f>
@@ -3340,10 +3340,10 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>9230000</v>
+        <v>3690000</v>
       </c>
       <c r="C14" s="12" t="n">
-        <v>9892700</v>
+        <v>4031925</v>
       </c>
       <c r="D14" s="12">
         <f>C14-B14</f>
@@ -3361,10 +3361,10 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>23500000</v>
+        <v>9400000</v>
       </c>
       <c r="C15" s="12" t="n">
-        <v>25310000</v>
+        <v>10043295</v>
       </c>
       <c r="D15" s="12">
         <f>C15-B15</f>
@@ -3447,7 +3447,7 @@
         </is>
       </c>
       <c r="B2" s="6" t="n">
-        <v>45.3</v>
+        <v>46.1</v>
       </c>
       <c r="C2" s="6" t="n">
         <v>45</v>
@@ -3472,10 +3472,10 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>58.1</v>
+        <v>59.8</v>
       </c>
       <c r="C3" s="6" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D3" s="14" t="n">
         <v>61</v>
@@ -3497,13 +3497,13 @@
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>39.2</v>
+        <v>38.5</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>34</v>
       </c>
       <c r="D4" s="14" t="n">
-        <v>34.1</v>
+        <v>34</v>
       </c>
       <c r="E4" s="15">
         <f>D4-C4</f>
@@ -3522,13 +3522,13 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>64.2</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D5" s="14" t="n">
-        <v>78.8</v>
+        <v>79</v>
       </c>
       <c r="E5" s="15">
         <f>D5-C5</f>
@@ -3548,10 +3548,10 @@
       </c>
       <c r="B6" s="6" t="n"/>
       <c r="C6" s="6" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D6" s="14" t="n">
-        <v>22.1</v>
+        <v>24.2</v>
       </c>
       <c r="E6" s="15">
         <f>D6-C6</f>
@@ -3571,10 +3571,10 @@
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D7" s="14" t="n">
-        <v>8.300000000000001</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="E7" s="15">
         <f>D7-C7</f>
@@ -3593,13 +3593,13 @@
         </is>
       </c>
       <c r="B8" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="C8" s="6" t="n">
         <v>1.45</v>
       </c>
-      <c r="C8" s="6" t="n">
-        <v>1.4</v>
-      </c>
       <c r="D8" s="14" t="n">
-        <v>1.8</v>
+        <v>1.63</v>
       </c>
       <c r="E8" s="15">
         <f>D8-C8</f>
@@ -3618,10 +3618,10 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>4.8</v>
+        <v>4.6</v>
       </c>
       <c r="C9" s="6" t="n">
-        <v>4.5</v>
+        <v>4.2</v>
       </c>
       <c r="D9" s="14" t="n">
         <v>3.6</v>
@@ -3679,23 +3679,23 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>3300000</v>
+        <v>1440000</v>
       </c>
       <c r="C2" s="12" t="n">
-        <v>3300000</v>
+        <v>1440000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>Efecto volumen (margen std 24%)</t>
+          <t>Efecto volumen (margen std 26%)</t>
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>-264000</v>
+        <v>-117000</v>
       </c>
       <c r="C3" s="9" t="n">
-        <v>3036000</v>
+        <v>1323000</v>
       </c>
     </row>
     <row r="4">
@@ -3705,10 +3705,10 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>-144000</v>
+        <v>-65000</v>
       </c>
       <c r="C4" s="9" t="n">
-        <v>2892000</v>
+        <v>1258000</v>
       </c>
     </row>
     <row r="5">
@@ -3718,10 +3718,10 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>-300000</v>
+        <v>-120000</v>
       </c>
       <c r="C5" s="9" t="n">
-        <v>2592000</v>
+        <v>1138000</v>
       </c>
     </row>
     <row r="6">
@@ -3731,10 +3731,10 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>-239600</v>
+        <v>-83400</v>
       </c>
       <c r="C6" s="9" t="n">
-        <v>2352400</v>
+        <v>1054600</v>
       </c>
     </row>
     <row r="7">
@@ -3744,10 +3744,10 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>-2400</v>
+        <v>-4600</v>
       </c>
       <c r="C7" s="9" t="n">
-        <v>2350000</v>
+        <v>1050000</v>
       </c>
     </row>
     <row r="8">
@@ -3757,10 +3757,10 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>2350000</v>
+        <v>1050000</v>
       </c>
       <c r="C8" s="12" t="n">
-        <v>2350000</v>
+        <v>1050000</v>
       </c>
     </row>
   </sheetData>
@@ -3813,7 +3813,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>662700</v>
+        <v>341925</v>
       </c>
       <c r="C3" s="6" t="n"/>
     </row>
@@ -3824,7 +3824,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>450000</v>
+        <v>180000</v>
       </c>
       <c r="C4" s="6" t="n"/>
     </row>
@@ -3835,7 +3835,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>-1360000</v>
+        <v>-526400</v>
       </c>
       <c r="C5" s="6" t="n"/>
     </row>
@@ -3846,7 +3846,7 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>-800000</v>
+        <v>-226895</v>
       </c>
       <c r="C6" s="6" t="n"/>
     </row>
@@ -3857,7 +3857,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>-180000</v>
+        <v>-148300</v>
       </c>
       <c r="C7" s="6" t="n"/>
     </row>
@@ -3868,7 +3868,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>100000</v>
+        <v>40000</v>
       </c>
       <c r="C8" s="6" t="n"/>
     </row>
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>-1127300</v>
+        <v>-339670</v>
       </c>
       <c r="C9" s="6">
         <f>SUM(B3:B8)</f>
@@ -3893,7 +3893,7 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>-350000</v>
+        <v>-170000</v>
       </c>
       <c r="C10" s="6" t="n"/>
     </row>
@@ -3904,7 +3904,7 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>2297300</v>
+        <v>839670</v>
       </c>
       <c r="C11" s="6" t="n"/>
     </row>
@@ -3915,7 +3915,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>-1070000</v>
+        <v>-430000</v>
       </c>
       <c r="C12" s="6" t="n"/>
     </row>
@@ -3926,7 +3926,7 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>-250000</v>
+        <v>-100000</v>
       </c>
       <c r="C13" s="6">
         <f>B9+B10+B11+B12+B13</f>
@@ -3999,7 +3999,7 @@
         </is>
       </c>
       <c r="B3" s="9" t="n">
-        <v>10400000</v>
+        <v>4100000</v>
       </c>
     </row>
     <row r="4">
@@ -4009,7 +4009,7 @@
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>10700000</v>
+        <v>4300000</v>
       </c>
     </row>
     <row r="5">
@@ -4019,7 +4019,7 @@
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>10900000</v>
+        <v>4400000</v>
       </c>
     </row>
     <row r="6">
@@ -4029,7 +4029,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>11200000</v>
+        <v>4500000</v>
       </c>
     </row>
     <row r="7">
@@ -4039,7 +4039,7 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>10600000</v>
+        <v>4200000</v>
       </c>
     </row>
     <row r="8">
@@ -4049,7 +4049,7 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>10000000</v>
+        <v>4000000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>